<commit_message>
Portfolio Yield Analysis v7: Loss Rate header alignment; METHODS/tracker v37/README
</commit_message>
<xml_diff>
--- a/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261028_v7_DRAFT.xlsx
+++ b/Prior Responses (outside data room)/Zed Portfolio Yield Analysis_20261028_v7_DRAFT.xlsx
@@ -90,7 +90,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="30">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -127,9 +127,6 @@
     </xf>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="10" fontId="4" fillId="4" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -2625,42 +2622,42 @@
     </row>
     <row r="3"/>
     <row r="4" ht="48" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
+      <c r="A4" s="5" t="inlineStr">
         <is>
           <t>Origination month</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B4" s="6" t="inlineStr">
         <is>
           <t>Accounts</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="C4" s="6" t="inlineStr">
         <is>
           <t>Principal originated</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D4" s="6" t="inlineStr">
         <is>
           <t>Seasoned principal (due ≥90 days ago)</t>
         </is>
       </c>
-      <c r="E4" s="24" t="inlineStr">
+      <c r="E4" s="6" t="inlineStr">
         <is>
           <t>Excluded: FPD principal 90+ DPD</t>
         </is>
       </c>
-      <c r="F4" s="24" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>Denominator: seasoned, ex-FPD</t>
         </is>
       </c>
-      <c r="G4" s="24" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>Numerator: 90+ DPD, ex-FPD</t>
         </is>
       </c>
-      <c r="H4" s="24" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>Loss rate</t>
         </is>
@@ -2957,14 +2954,14 @@
         <f>SUM(G5:G13)</f>
         <v/>
       </c>
-      <c r="H14" s="25">
+      <c r="H14" s="24">
         <f>G14/F14</f>
         <v/>
       </c>
     </row>
     <row r="15"/>
     <row r="16" ht="15" customHeight="1">
-      <c r="A16" s="26" t="inlineStr">
+      <c r="A16" s="25" t="inlineStr">
         <is>
           <t>How to read this table</t>
         </is>
@@ -3061,22 +3058,22 @@
           <t>Jan 2026</t>
         </is>
       </c>
-      <c r="B24" s="27" t="n">
+      <c r="B24" s="26" t="n">
         <v>0.00675</v>
       </c>
-      <c r="C24" s="27" t="n">
+      <c r="C24" s="26" t="n">
         <v>0.02263</v>
       </c>
-      <c r="D24" s="27" t="n">
+      <c r="D24" s="26" t="n">
         <v>0.02263</v>
       </c>
-      <c r="E24" s="27" t="n">
+      <c r="E24" s="26" t="n">
         <v>0.02263</v>
       </c>
-      <c r="F24" s="27" t="n">
+      <c r="F24" s="26" t="n">
         <v>0.02263</v>
       </c>
-      <c r="G24" s="28" t="n">
+      <c r="G24" s="27" t="n">
         <v>0.02263</v>
       </c>
       <c r="H24" t="n">
@@ -3089,24 +3086,24 @@
           <t>Feb 2026</t>
         </is>
       </c>
-      <c r="B25" s="27" t="n">
+      <c r="B25" s="26" t="n">
         <v>0.00851</v>
       </c>
-      <c r="C25" s="27" t="n">
+      <c r="C25" s="26" t="n">
         <v>0.01028</v>
       </c>
-      <c r="D25" s="27" t="n">
+      <c r="D25" s="26" t="n">
         <v>0.01118</v>
       </c>
-      <c r="E25" s="27" t="n">
+      <c r="E25" s="26" t="n">
         <v>0.01128</v>
       </c>
-      <c r="F25" s="27" t="inlineStr">
+      <c r="F25" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G25" s="28" t="n">
+      <c r="G25" s="27" t="n">
         <v>0.01128</v>
       </c>
       <c r="H25" t="n">
@@ -3119,24 +3116,24 @@
           <t>Mar 2026</t>
         </is>
       </c>
-      <c r="B26" s="27" t="n">
+      <c r="B26" s="26" t="n">
         <v>0.00455</v>
       </c>
-      <c r="C26" s="27" t="n">
+      <c r="C26" s="26" t="n">
         <v>0.01469</v>
       </c>
-      <c r="D26" s="27" t="n">
+      <c r="D26" s="26" t="n">
         <v>0.01577</v>
       </c>
-      <c r="E26" s="27" t="n">
+      <c r="E26" s="26" t="n">
         <v>0.01577</v>
       </c>
-      <c r="F26" s="27" t="inlineStr">
+      <c r="F26" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G26" s="28" t="n">
+      <c r="G26" s="27" t="n">
         <v>0.01577</v>
       </c>
       <c r="H26" t="n">
@@ -3149,26 +3146,26 @@
           <t>Apr 2026</t>
         </is>
       </c>
-      <c r="B27" s="27" t="n">
+      <c r="B27" s="26" t="n">
         <v>0.00773</v>
       </c>
-      <c r="C27" s="27" t="n">
+      <c r="C27" s="26" t="n">
         <v>0.01313</v>
       </c>
-      <c r="D27" s="27" t="n">
+      <c r="D27" s="26" t="n">
         <v>0.01366</v>
       </c>
-      <c r="E27" s="27" t="inlineStr">
+      <c r="E27" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F27" s="27" t="inlineStr">
+      <c r="F27" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G27" s="28" t="n">
+      <c r="G27" s="27" t="n">
         <v>0.01386</v>
       </c>
       <c r="H27" t="n">
@@ -3181,28 +3178,28 @@
           <t>May 2026</t>
         </is>
       </c>
-      <c r="B28" s="27" t="n">
+      <c r="B28" s="26" t="n">
         <v>0.00494</v>
       </c>
-      <c r="C28" s="27" t="n">
+      <c r="C28" s="26" t="n">
         <v>0.00758</v>
       </c>
-      <c r="D28" s="27" t="inlineStr">
+      <c r="D28" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E28" s="27" t="inlineStr">
+      <c r="E28" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F28" s="27" t="inlineStr">
+      <c r="F28" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G28" s="28" t="n">
+      <c r="G28" s="27" t="n">
         <v>0.00906</v>
       </c>
       <c r="H28" t="n">
@@ -3215,30 +3212,30 @@
           <t>Jun 2026</t>
         </is>
       </c>
-      <c r="B29" s="27" t="n">
+      <c r="B29" s="26" t="n">
         <v>0.00215</v>
       </c>
-      <c r="C29" s="27" t="inlineStr">
+      <c r="C29" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D29" s="27" t="inlineStr">
+      <c r="D29" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="E29" s="27" t="inlineStr">
+      <c r="E29" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="F29" s="27" t="inlineStr">
+      <c r="F29" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="G29" s="28" t="n">
+      <c r="G29" s="27" t="n">
         <v>0.00338</v>
       </c>
       <c r="H29" t="n">
@@ -3246,7 +3243,7 @@
       </c>
     </row>
     <row r="30" ht="15" customHeight="1">
-      <c r="A30" s="26" t="inlineStr">
+      <c r="A30" s="25" t="inlineStr">
         <is>
           <t>How to read this table</t>
         </is>
@@ -3323,7 +3320,7 @@
       </c>
     </row>
     <row r="4" ht="75" customHeight="1">
-      <c r="A4" s="29" t="inlineStr">
+      <c r="A4" s="28" t="inlineStr">
         <is>
           <t>Scope</t>
         </is>
@@ -3335,7 +3332,7 @@
       </c>
     </row>
     <row r="5" ht="195" customHeight="1">
-      <c r="A5" s="29" t="inlineStr">
+      <c r="A5" s="28" t="inlineStr">
         <is>
           <t>Book month (yield basis)</t>
         </is>
@@ -3347,7 +3344,7 @@
       </c>
     </row>
     <row r="6" ht="30" customHeight="1">
-      <c r="A6" s="29" t="inlineStr">
+      <c r="A6" s="28" t="inlineStr">
         <is>
           <t>Annualization</t>
         </is>
@@ -3359,7 +3356,7 @@
       </c>
     </row>
     <row r="7" ht="105" customHeight="1">
-      <c r="A7" s="29" t="inlineStr">
+      <c r="A7" s="28" t="inlineStr">
         <is>
           <t>Revolving interest</t>
         </is>
@@ -3371,7 +3368,7 @@
       </c>
     </row>
     <row r="8" ht="105" customHeight="1">
-      <c r="A8" s="29" t="inlineStr">
+      <c r="A8" s="28" t="inlineStr">
         <is>
           <t>Installment interest and upfront fees</t>
         </is>
@@ -3383,7 +3380,7 @@
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
-      <c r="A9" s="29" t="inlineStr">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Late payment fees</t>
         </is>
@@ -3395,7 +3392,7 @@
       </c>
     </row>
     <row r="10" ht="90" customHeight="1">
-      <c r="A10" s="29" t="inlineStr">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t>Interchange</t>
         </is>
@@ -3407,7 +3404,7 @@
       </c>
     </row>
     <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="29" t="inlineStr">
+      <c r="A11" s="28" t="inlineStr">
         <is>
           <t>Turnover</t>
         </is>
@@ -3419,7 +3416,7 @@
       </c>
     </row>
     <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="29" t="inlineStr">
+      <c r="A12" s="28" t="inlineStr">
         <is>
           <t>Principal flow</t>
         </is>
@@ -3431,7 +3428,7 @@
       </c>
     </row>
     <row r="13" ht="90" customHeight="1">
-      <c r="A13" s="29" t="inlineStr">
+      <c r="A13" s="28" t="inlineStr">
         <is>
           <t>Principal originated (Loss Rate tab)</t>
         </is>
@@ -3443,7 +3440,7 @@
       </c>
     </row>
     <row r="14" ht="90" customHeight="1">
-      <c r="A14" s="29" t="inlineStr">
+      <c r="A14" s="28" t="inlineStr">
         <is>
           <t>Loss rate</t>
         </is>
@@ -3455,7 +3452,7 @@
       </c>
     </row>
     <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="29" t="inlineStr">
+      <c r="A15" s="28" t="inlineStr">
         <is>
           <t>Loss on receivables</t>
         </is>
@@ -3467,7 +3464,7 @@
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
-      <c r="A16" s="29" t="inlineStr">
+      <c r="A16" s="28" t="inlineStr">
         <is>
           <t>Net yield</t>
         </is>
@@ -3479,7 +3476,7 @@
       </c>
     </row>
     <row r="17" ht="75" customHeight="1">
-      <c r="A17" s="29" t="inlineStr">
+      <c r="A17" s="28" t="inlineStr">
         <is>
           <t>Sources</t>
         </is>
@@ -3491,7 +3488,7 @@
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
-      <c r="A18" s="29" t="inlineStr">
+      <c r="A18" s="28" t="inlineStr">
         <is>
           <t>Prepared</t>
         </is>

</xml_diff>